<commit_message>
Auto update CodeMetrix trackers
</commit_message>
<xml_diff>
--- a/Students.xlsx
+++ b/Students.xlsx
@@ -5624,17 +5624,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>922525106036</t>
+          <t>922525106027</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>BALARITHISH S</t>
+          <t>Arulesh K</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>arul2008</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -5644,24 +5644,24 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/3/</t>
+          <t>https://leetcode.com/u/arul2008/</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>922525106035</t>
+          <t>922525106036</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>BALAJI C</t>
+          <t>BALARITHISH S</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -5671,24 +5671,24 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/4/</t>
+          <t>https://leetcode.com/u/3/</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>922525106058</t>
+          <t>922525106035</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>DEEKSHA K</t>
+          <t>BALAJI C</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -5698,24 +5698,24 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/5/</t>
+          <t>https://leetcode.com/u/4/</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>922525106011</t>
+          <t>922525106058</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>AJAYKRISHNA R</t>
+          <t>DEEKSHA K</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>922525106011</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -5725,24 +5725,24 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/922525106011/</t>
+          <t>https://leetcode.com/u/5/</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>922525106049</t>
+          <t>922525106011</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>BUVNESH N</t>
+          <t>AJAYKRISHNA R</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>922525106049</t>
+          <t>922525106011</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -5752,24 +5752,24 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/922525106049/</t>
+          <t>https://leetcode.com/u/922525106011/</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>922525106052</t>
+          <t>922525106049</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>CHINMAYASRI K</t>
+          <t>BUVNESH N</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>922525106052</t>
+          <t>922525106049</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -5779,24 +5779,24 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/922525106052/</t>
+          <t>https://leetcode.com/u/922525106049/</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>922525106055</t>
+          <t>922525106052</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>DARSHAN C</t>
+          <t>CHINMAYASRI K</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>922525106055</t>
+          <t>922525106052</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -5806,51 +5806,51 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/922525106055/</t>
+          <t>https://leetcode.com/u/922525106052/</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>922525106093</t>
+          <t>922525106055</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>GIRIVASH P</t>
+          <t>DARSHAN C</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>922525106093</t>
+          <t>922525106055</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>ECE B</t>
+          <t>ECE A</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/922525106093/</t>
+          <t>https://leetcode.com/u/922525106055/</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>922525106096</t>
+          <t>922525106093</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>GOPALA KRISHNAN C</t>
+          <t>GIRIVASH P</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>922525106096</t>
+          <t>922525106093</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -5860,24 +5860,24 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/922525106096/</t>
+          <t>https://leetcode.com/u/922525106093/</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>922525106097</t>
+          <t>922525106096</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>GOPINATH R</t>
+          <t>GOPALA KRISHNAN C</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>922525106097</t>
+          <t>922525106096</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -5887,51 +5887,51 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/922525106097/</t>
+          <t>https://leetcode.com/u/922525106096/</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>922525106056</t>
+          <t>922525106097</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>DARSHAN MANISH A</t>
+          <t>GOPINATH R</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2007darshan</t>
+          <t>922525106097</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>ECE A</t>
+          <t>ECE B</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/2007darshan/</t>
+          <t>https://leetcode.com/u/922525106097/</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>922525106006</t>
+          <t>922525106056</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>AFTON AJ</t>
+          <t>DARSHAN MANISH A</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>afton_2008</t>
+          <t>2007darshan</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -5941,24 +5941,24 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/afton_2008/</t>
+          <t>https://leetcode.com/u/2007darshan/</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>922525106028</t>
+          <t>922525106006</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>ARUN C</t>
+          <t>AFTON AJ</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>AGmXRQ1yTe</t>
+          <t>afton_2008</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -5968,24 +5968,24 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/AGmXRQ1yTe/</t>
+          <t>https://leetcode.com/u/afton_2008/</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>922525106013</t>
+          <t>922525106028</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>AJITH KUMAR M</t>
+          <t>ARUN C</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>ajit_kumar_23</t>
+          <t>AGmXRQ1yTe</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -5995,24 +5995,24 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/ajit_kumar_23/</t>
+          <t>https://leetcode.com/u/AGmXRQ1yTe/</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>922525106019</t>
+          <t>922525106013</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>ANBARASU S</t>
+          <t>AJITH KUMAR M</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Anbarasu28122007</t>
+          <t>ajit_kumar_23</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -6022,24 +6022,24 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Anbarasu28122007/</t>
+          <t>https://leetcode.com/u/ajit_kumar_23/</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>922525106021</t>
+          <t>922525106020</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>ANOOP C</t>
+          <t>ANJITHAA N</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>anoop_appuz</t>
+          <t>Anjithaa2006</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -6049,24 +6049,24 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/anoop_appuz/</t>
+          <t>https://leetcode.com/u/Anjithaa2006/</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>922525106022</t>
+          <t>922525106021</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>ANUJA S</t>
+          <t>ANOOP C</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>anuja008</t>
+          <t>anoop_appuz</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -6076,24 +6076,24 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/anuja008/</t>
+          <t>https://leetcode.com/u/anoop_appuz/</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>922525106027</t>
+          <t>922525106022</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Arulesh K</t>
+          <t>ANUJA S</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>arul2008</t>
+          <t>anuja008</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -6103,7 +6103,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/arul2008/</t>
+          <t>https://leetcode.com/u/anuja008/</t>
         </is>
       </c>
     </row>
@@ -6893,17 +6893,17 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>922525106020</t>
+          <t>922525106019</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>ANJITHAA N</t>
+          <t>ANBARASU S</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Anjithaa2006</t>
+          <t>Anbarasu28122007</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -6913,7 +6913,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>https://leetcode.com/u/Anjithaa2006/</t>
+          <t>https://leetcode.com/u/Anbarasu28122007/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove blank ghost student entry, resolve merge conflict rows, and sanitize dataset across CSV and tracker files
</commit_message>
<xml_diff>
--- a/Students.xlsx
+++ b/Students.xlsx
@@ -1,17 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Students" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Students" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Students'!$A$1:$E$369</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -29,23 +27,17 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002563EB"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -53,14 +45,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -427,15 +425,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E369"/>
+  <dimension ref="A1:D369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -458,11 +449,6 @@
           <t>Section</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>LeetCode Link</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -485,11 +471,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/saran32/</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -512,11 +493,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/dharshinideivasigamani/</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -539,11 +515,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/santhosh7811/</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -566,11 +537,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/X01u2FNNX4/</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -593,11 +559,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sabareesh_karikalan/</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -620,11 +581,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/8925787430/</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -647,11 +603,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/GSIVANESH/</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -674,11 +625,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sivagnanam3344/</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -701,11 +647,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Rithanya12-3/</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -728,11 +669,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Rithika_Balakrishnan/</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -755,11 +691,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/RohithrohiV/</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -782,11 +713,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Roobagapriya/</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -809,11 +735,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sivaprakash_0406/</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -836,11 +757,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/9043374912/</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -863,11 +779,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Shree_Harini478/</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -890,11 +801,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/itsmesanjay007/</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -917,11 +823,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/shivani208/</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -944,11 +845,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sharath_1010/</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -971,11 +867,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/ShanthiniChelladurai/</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -998,11 +889,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/shahana_pandiraj04/</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1025,11 +911,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sivanesh2007/</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1052,11 +933,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Jna76WrjNd/</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1079,11 +955,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Senthamizh08/</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1106,11 +977,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/SanjayUdayan/</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1133,11 +999,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Selvax07/</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1160,11 +1021,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/santhoshsathya260/</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1187,11 +1043,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sarvesh312008/</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1214,11 +1065,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Rithik_78/</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1241,11 +1087,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Rithish_/</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1268,11 +1109,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Sahanavijayakumar_0033/</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1295,11 +1131,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sakthivel23116/</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1322,11 +1153,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/saswin_88/</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1349,11 +1175,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Selvapragadeesh/</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1376,11 +1197,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Selvakumarsk-32/</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1403,11 +1219,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sashmikaprabhu/</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1430,11 +1241,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/shreecharan22/</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1457,11 +1263,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sarika_5408/</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1484,11 +1285,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/roshan2403/</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1511,11 +1307,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/roshikaveeramalai/</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1538,11 +1329,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Rubesh_7/</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1565,11 +1351,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/SabarivasanP/</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1592,11 +1373,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Saravanan_7525/</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1619,11 +1395,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Sakthisaro08/</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1646,11 +1417,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/saravanan__k__/</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1673,11 +1439,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sandhosh_30_R/</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1700,11 +1461,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sanjay00675/</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1727,11 +1483,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sanmathi06/</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1754,11 +1505,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/santhiya0202/</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1781,11 +1527,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/santhosh2407/</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1808,11 +1549,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/santhosh8760/</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1835,11 +1571,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Sethupathi_1228/</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1862,11 +1593,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/itz__priyan__/</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1889,11 +1615,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/velliangiri_R/</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1916,11 +1637,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/O8bYDSRUbE/</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1943,11 +1659,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/VIGNESHWAR0221/</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1970,11 +1681,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/vijayaragavan1216/</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1997,11 +1703,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/vikramvicky5678/</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2024,11 +1725,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/VISHNU_B_2008/</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2051,11 +1747,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Vishnuharan082007/</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2078,11 +1769,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/_swathi_3366/</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2105,11 +1791,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sujith45/</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2132,11 +1813,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/thirishavsb/</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2159,11 +1835,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Swetha_20_1/</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2186,11 +1857,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/vishnupriyamaran/</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2213,11 +1879,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/VISU_YAZHU/</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2240,11 +1901,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Vicky_27_Velan/</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2267,11 +1923,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/vishwajeth/</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2294,11 +1945,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/THIRINESHKUMAR0608/</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2321,11 +1967,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/yaswanth_2008/</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2348,11 +1989,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/yazhini2007/</t>
-        </is>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2375,11 +2011,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/SIVARANJAN_MP/</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2402,11 +2033,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Sivasanjeev16/</t>
-        </is>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2429,11 +2055,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/AK_Siva/</t>
-        </is>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2456,11 +2077,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sivatharun22/</t>
-        </is>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2483,11 +2099,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/_sobika_R/</t>
-        </is>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2510,11 +2121,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/SREEDHARANI_14/</t>
-        </is>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2537,11 +2143,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/yazhini__1234/</t>
-        </is>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2564,11 +2165,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Yashnisubramaniyan/</t>
-        </is>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2591,11 +2187,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/syokeswaran/</t>
-        </is>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2618,11 +2209,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Sri1540/</t>
-        </is>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2645,11 +2231,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sriheera03/</t>
-        </is>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2672,11 +2253,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/kanth2008/</t>
-        </is>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2699,11 +2275,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Srisastika_1401/</t>
-        </is>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2726,11 +2297,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/srivarshan_B_P/</t>
-        </is>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2753,11 +2319,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/V_SRINATH/</t>
-        </is>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2780,11 +2341,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/SRINIRANJAN2008/</t>
-        </is>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2807,11 +2363,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/srinithe_1401/</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2834,11 +2385,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Srinithi24_/</t>
-        </is>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2861,11 +2407,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/mahi/</t>
-        </is>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2888,11 +2429,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Subarna_17/</t>
-        </is>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2915,11 +2451,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/subika1112/</t>
-        </is>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2942,11 +2473,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Sudharsan/</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2969,11 +2495,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/SUGANTHKALAI/</t>
-        </is>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2996,11 +2517,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Sugi_07/</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3023,11 +2539,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/SUJEETH77/</t>
-        </is>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3050,11 +2561,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sumithra_16/</t>
-        </is>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3077,11 +2583,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/surya001prabhu/</t>
-        </is>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3104,11 +2605,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Susidharan147/</t>
-        </is>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3131,11 +2627,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sutharshana743/</t>
-        </is>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3158,11 +2649,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Swathimanivel_1234/</t>
-        </is>
-      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3185,11 +2671,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Kdmif0HMNm/</t>
-        </is>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3212,11 +2693,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/thamarai_04/</t>
-        </is>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3239,11 +2715,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Thameem_786/</t>
-        </is>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3266,11 +2737,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/THARANISH2008/</t>
-        </is>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3293,11 +2759,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Tharunika_12/</t>
-        </is>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3320,11 +2781,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/thiru0211_/</t>
-        </is>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3347,11 +2803,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/vaish200/</t>
-        </is>
-      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3374,11 +2825,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/VASANTH2007/</t>
-        </is>
-      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3401,11 +2847,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/_vasanth_s_/</t>
-        </is>
-      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3428,11 +2869,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Vasanthakumar12232/</t>
-        </is>
-      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3455,11 +2891,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/VasanthKumar008/</t>
-        </is>
-      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3482,11 +2913,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/GTVASU2008/</t>
-        </is>
-      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3509,11 +2935,6 @@
           <t>ECE F</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/vasuki/</t>
-        </is>
-      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3536,11 +2957,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/SAJISH7/</t>
-        </is>
-      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3563,11 +2979,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/zklXTc9UAp/</t>
-        </is>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3590,11 +3001,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sanjayan31/</t>
-        </is>
-      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3617,11 +3023,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Sathana-1267/</t>
-        </is>
-      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3644,11 +3045,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/shandoshsai/</t>
-        </is>
-      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3671,11 +3067,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sharukesh2008/</t>
-        </is>
-      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3698,11 +3089,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/krish-2007/</t>
-        </is>
-      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3725,11 +3111,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/itz_lakshe/</t>
-        </is>
-      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3752,11 +3133,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/lavilavanya/</t>
-        </is>
-      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3779,11 +3155,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/LING2007/</t>
-        </is>
-      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3806,11 +3177,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/LogadharshiniT/</t>
-        </is>
-      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3833,11 +3199,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Loga07/</t>
-        </is>
-      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3860,11 +3221,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/loga16/</t>
-        </is>
-      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3887,11 +3243,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/LOGESHWARAN2008/</t>
-        </is>
-      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3914,11 +3265,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/LOHITH012008/</t>
-        </is>
-      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -3941,11 +3287,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/LOKRAJI6793/</t>
-        </is>
-      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -3968,11 +3309,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/jenita0206/</t>
-        </is>
-      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -3995,11 +3331,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Madhankumar861053/</t>
-        </is>
-      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4022,11 +3353,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/madhudhara/</t>
-        </is>
-      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4049,11 +3375,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Madhumitha42/</t>
-        </is>
-      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4076,11 +3397,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Madhupkishor_20/</t>
-        </is>
-      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4103,11 +3419,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/mahalakshmi182025/</t>
-        </is>
-      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4130,11 +3441,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/maha_lakh_20/</t>
-        </is>
-      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4157,11 +3463,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Mahinabhishek0411/</t>
-        </is>
-      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4184,11 +3485,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/manishaa_20/</t>
-        </is>
-      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4211,11 +3507,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Manoj_1319/</t>
-        </is>
-      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -4238,11 +3529,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/m____a____n____o____/</t>
-        </is>
-      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -4265,11 +3551,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/mathesh25/</t>
-        </is>
-      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -4292,11 +3573,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Mayakannan129/</t>
-        </is>
-      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -4319,11 +3595,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Mayuka_M/</t>
-        </is>
-      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4346,11 +3617,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/milan190308/</t>
-        </is>
-      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -4373,11 +3639,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/itsmoni/</t>
-        </is>
-      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -4400,11 +3661,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Monishav2007/</t>
-        </is>
-      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -4427,11 +3683,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/morrishd/</t>
-        </is>
-      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -4454,11 +3705,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Mouleeshwari2008/</t>
-        </is>
-      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -4481,11 +3727,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Moushmi_20/</t>
-        </is>
-      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -4508,11 +3749,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/mythilimurugesan/</t>
-        </is>
-      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -4535,11 +3771,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/NafreenJohnbasha/</t>
-        </is>
-      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -4562,11 +3793,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/nandhini546/</t>
-        </is>
-      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -4589,11 +3815,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/lnavaneethan08/</t>
-        </is>
-      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -4616,11 +3837,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/NAVEETHAN/</t>
-        </is>
-      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -4643,11 +3859,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/niranjani_123/</t>
-        </is>
-      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -4670,11 +3881,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Nithishct123/</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -4697,11 +3903,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Nithish_P_CS/</t>
-        </is>
-      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -4724,11 +3925,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/nithishramalingam007/</t>
-        </is>
-      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -4751,11 +3947,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E160" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/nithishwaran25/</t>
-        </is>
-      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -4778,11 +3969,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E161" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/NithyashreeG10/</t>
-        </is>
-      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -4805,11 +3991,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Nithyashree273/</t>
-        </is>
-      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -4832,11 +4013,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E163" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Nithyasri2008/</t>
-        </is>
-      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -4859,11 +4035,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E164" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/paargavi2007/</t>
-        </is>
-      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -4886,11 +4057,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E165" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/pavithra145/</t>
-        </is>
-      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -4913,11 +4079,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E166" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Pavithran_S_/</t>
-        </is>
-      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -4940,11 +4101,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E167" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Piraveen2025/</t>
-        </is>
-      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -4967,11 +4123,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E168" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/_d_Prabhakaran_/</t>
-        </is>
-      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -4994,11 +4145,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E169" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/pradhosh/</t>
-        </is>
-      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -5021,11 +4167,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E170" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/pragalathan070108/</t>
-        </is>
-      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -5048,11 +4189,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E171" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Pranesh-Y/</t>
-        </is>
-      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -5075,11 +4211,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E172" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/pranithaashree/</t>
-        </is>
-      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -5102,11 +4233,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E173" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/praveen1247/</t>
-        </is>
-      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -5129,11 +4255,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/praveen_3208/</t>
-        </is>
-      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -5156,11 +4277,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E175" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/PRAVEENGANESAN/</t>
-        </is>
-      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -5183,11 +4299,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E176" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/itz_praveen_/</t>
-        </is>
-      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -5210,11 +4321,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E177" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/preethy2007/</t>
-        </is>
-      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -5237,11 +4343,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E178" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/prithiv16/</t>
-        </is>
-      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -5264,11 +4365,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E179" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/priyadharshini1551/</t>
-        </is>
-      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -5291,11 +4387,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E180" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Priyankaashok1201/</t>
-        </is>
-      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -5318,11 +4409,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/priyankadhanush23/</t>
-        </is>
-      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -5345,11 +4431,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E182" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Ragadharshini_2181/</t>
-        </is>
-      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -5372,11 +4453,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E183" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/ragunath24/</t>
-        </is>
-      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -5399,11 +4475,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E184" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/rahulkajan/</t>
-        </is>
-      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -5426,11 +4497,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E185" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/rajaprahadeeswaran/</t>
-        </is>
-      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -5453,11 +4519,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E186" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/RANJANA_2007/</t>
-        </is>
-      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -5480,11 +4541,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E187" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/RASIKA_2008/</t>
-        </is>
-      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -5507,11 +4563,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E188" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Rathish2025/</t>
-        </is>
-      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -5534,11 +4585,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E189" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Ravikumar_14/</t>
-        </is>
-      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -5561,11 +4607,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E190" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/logesh2008/</t>
-        </is>
-      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -5588,11 +4629,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E191" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/ADHITHMITHRAN/</t>
-        </is>
-      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -5615,11 +4651,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E192" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/2/</t>
-        </is>
-      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -5642,11 +4673,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E193" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/arul2008/</t>
-        </is>
-      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -5669,11 +4695,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E194" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Bharanidharan_2007/</t>
-        </is>
-      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -5696,11 +4717,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E195" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/3/</t>
-        </is>
-      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -5723,11 +4739,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E196" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/4/</t>
-        </is>
-      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -5750,11 +4761,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E197" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/5/</t>
-        </is>
-      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -5777,11 +4783,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E198" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106011/</t>
-        </is>
-      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -5804,11 +4805,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E199" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106049/</t>
-        </is>
-      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -5831,11 +4827,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E200" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106052/</t>
-        </is>
-      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -5858,11 +4849,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106055/</t>
-        </is>
-      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -5885,11 +4871,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E202" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106093/</t>
-        </is>
-      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -5912,11 +4893,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E203" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106096/</t>
-        </is>
-      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -5939,11 +4915,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E204" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106097/</t>
-        </is>
-      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -5966,11 +4937,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E205" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/2007darshan/</t>
-        </is>
-      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -5993,11 +4959,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E206" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/afton_2008/</t>
-        </is>
-      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -6020,11 +4981,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E207" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/AGmXRQ1yTe/</t>
-        </is>
-      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -6047,11 +5003,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E208" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/ajit_kumar_23/</t>
-        </is>
-      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -6074,11 +5025,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E209" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Anbarasu28122007/</t>
-        </is>
-      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -6101,11 +5047,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E210" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Anjithaa2006/</t>
-        </is>
-      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -6128,11 +5069,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E211" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/anoop_appuz/</t>
-        </is>
-      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -6155,11 +5091,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E212" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/anuja008/</t>
-        </is>
-      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -6182,11 +5113,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E213" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/B/</t>
-        </is>
-      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -6209,11 +5135,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E214" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/barani_7/</t>
-        </is>
-      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -6236,11 +5157,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E215" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Benov_18/</t>
-        </is>
-      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -6263,11 +5179,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E216" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/BhavanBala/</t>
-        </is>
-      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -6290,11 +5201,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E217" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/BK5226221/</t>
-        </is>
-      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -6317,11 +5223,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E218" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Boobase/</t>
-        </is>
-      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -6344,11 +5245,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E219" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/boomikat123/</t>
-        </is>
-      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -6371,11 +5267,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E220" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/BosviyaBSV/</t>
-        </is>
-      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -6398,11 +5289,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E221" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Brindha_S/</t>
-        </is>
-      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -6425,11 +5311,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E222" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/AkashRajaram/</t>
-        </is>
-      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -6452,11 +5333,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E223" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/charu120108/</t>
-        </is>
-      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -6479,11 +5355,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E224" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/charunethra07/</t>
-        </is>
-      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -6506,11 +5377,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E225" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/codewithakshaya/</t>
-        </is>
-      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -6533,11 +5399,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E226" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/codewithakshaya78/</t>
-        </is>
-      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -6560,11 +5421,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E227" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Dakshinya555/</t>
-        </is>
-      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -6587,11 +5443,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E228" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Darshan_mainsh008/</t>
-        </is>
-      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -6614,11 +5465,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E229" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/dejasri/</t>
-        </is>
-      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -6641,11 +5487,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E230" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/jakabesj/</t>
-        </is>
-      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -6668,11 +5509,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E231" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/jasvanthram/</t>
-        </is>
-      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -6695,11 +5531,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E232" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/UJw4zUNnJJ/</t>
-        </is>
-      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -6722,11 +5553,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E233" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/S_T_Arul/</t>
-        </is>
-      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -6749,11 +5575,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E234" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/vsdharsini/</t>
-        </is>
-      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -6776,11 +5597,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E235" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/tharik25/</t>
-        </is>
-      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -6803,11 +5619,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/smonish777/</t>
-        </is>
-      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -6830,11 +5641,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E237" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Renofiya-2007/</t>
-        </is>
-      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -6857,11 +5663,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E238" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/reshmi2008/</t>
-        </is>
-      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -6884,11 +5685,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E239" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/rethanya38/</t>
-        </is>
-      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -6911,11 +5707,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E240" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Rethish_R/</t>
-        </is>
-      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -6938,11 +5729,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E241" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/aashifasahanaj/</t>
-        </is>
-      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -6965,11 +5751,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E242" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/AAZHIGA/</t>
-        </is>
-      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -6992,11 +5773,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E243" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Abinaya7095/</t>
-        </is>
-      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -7019,11 +5795,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E244" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/abirami8072/</t>
-        </is>
-      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -7046,11 +5817,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E245" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/agatheeswarank/</t>
-        </is>
-      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -7073,11 +5839,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E246" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/codewithaish/</t>
-        </is>
-      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -7100,11 +5861,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E247" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Akshara015/</t>
-        </is>
-      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -7127,11 +5883,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E248" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Alageshwaran2008/</t>
-        </is>
-      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -7154,11 +5905,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E249" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/amirda_varsini_2007/</t>
-        </is>
-      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -7181,11 +5927,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E250" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Anusri_2008/</t>
-        </is>
-      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -7208,11 +5949,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E251" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/ANUSYA_30/</t>
-        </is>
-      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -7235,11 +5971,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E252" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Arunravi1810/</t>
-        </is>
-      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -7262,11 +5993,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E253" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Arunkumar2008/</t>
-        </is>
-      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -7289,11 +6015,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E254" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/arunprasanth6435/</t>
-        </is>
-      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -7316,11 +6037,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E255" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Arvin/</t>
-        </is>
-      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -7343,11 +6059,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E256" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/ASHOKKUMAR18/</t>
-        </is>
-      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -7370,11 +6081,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E257" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/1/</t>
-        </is>
-      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -7397,11 +6103,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E258" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/BharathwajX/</t>
-        </is>
-      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -7424,11 +6125,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E259" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/chinnappanrajniselvi/</t>
-        </is>
-      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -7451,11 +6147,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E260" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/desmashalini/</t>
-        </is>
-      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -7478,11 +6169,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E261" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Devaece/</t>
-        </is>
-      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -7505,11 +6191,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E262" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Dhaksesh_Pranav_P/</t>
-        </is>
-      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -7532,11 +6213,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E263" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Dhanasri_r/</t>
-        </is>
-      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -7559,11 +6235,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E264" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106064/</t>
-        </is>
-      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -7586,11 +6257,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E265" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106065/</t>
-        </is>
-      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -7613,11 +6279,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E266" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106066/</t>
-        </is>
-      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -7640,11 +6301,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E267" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106067/</t>
-        </is>
-      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -7667,11 +6323,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E268" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/dharaneeshk/</t>
-        </is>
-      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -7694,11 +6345,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E269" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106069/</t>
-        </is>
-      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -7721,11 +6367,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E270" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106070/</t>
-        </is>
-      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -7748,11 +6389,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E271" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106071/</t>
-        </is>
-      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -7775,11 +6411,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E272" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106072/</t>
-        </is>
-      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -7802,11 +6433,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E273" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106073/</t>
-        </is>
-      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -7829,11 +6455,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E274" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Dharshini_74/</t>
-        </is>
-      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -7856,11 +6477,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E275" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106075/</t>
-        </is>
-      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -7883,11 +6499,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E276" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106077/</t>
-        </is>
-      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -7910,11 +6521,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E277" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106078/</t>
-        </is>
-      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -7937,11 +6543,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E278" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106079/</t>
-        </is>
-      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -7964,11 +6565,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E279" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/kathir__21/</t>
-        </is>
-      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -7991,11 +6587,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E280" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/DhivakarR/</t>
-        </is>
-      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -8018,11 +6609,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E281" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106081/</t>
-        </is>
-      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -8045,11 +6631,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E282" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106099/</t>
-        </is>
-      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -8072,11 +6653,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E283" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106106/</t>
-        </is>
-      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -8099,11 +6675,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E284" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Dinesh_106082/</t>
-        </is>
-      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -8126,11 +6697,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E285" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106083/</t>
-        </is>
-      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -8153,11 +6719,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E286" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106084/</t>
-        </is>
-      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -8180,11 +6741,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E287" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106085/</t>
-        </is>
-      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -8207,11 +6763,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E288" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/princess-nk/</t>
-        </is>
-      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -8234,11 +6785,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E289" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106087/</t>
-        </is>
-      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -8261,11 +6807,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E290" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106088/</t>
-        </is>
-      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -8288,11 +6829,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E291" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106089/</t>
-        </is>
-      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -8315,11 +6851,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E292" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106090/</t>
-        </is>
-      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -8342,11 +6873,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E293" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106091/</t>
-        </is>
-      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -8369,11 +6895,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E294" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106092/</t>
-        </is>
-      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -8396,11 +6917,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E295" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Gokul_tamilan_india/</t>
-        </is>
-      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -8423,11 +6939,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E296" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/gomathi_0709/</t>
-        </is>
-      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -8450,11 +6961,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E297" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106098/</t>
-        </is>
-      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -8477,11 +6983,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E298" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106100/</t>
-        </is>
-      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -8504,11 +7005,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E299" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922524106101/</t>
-        </is>
-      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -8531,11 +7027,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E300" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106106/</t>
-        </is>
-      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -8558,11 +7049,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E301" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106103/</t>
-        </is>
-      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -8585,11 +7071,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E302" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106104/</t>
-        </is>
-      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -8612,11 +7093,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E303" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Gowtham_080/</t>
-        </is>
-      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -8639,11 +7115,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E304" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Gunashree20/</t>
-        </is>
-      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -8666,11 +7137,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E305" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106108/</t>
-        </is>
-      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -8693,11 +7159,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E306" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106109/</t>
-        </is>
-      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -8720,11 +7181,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E307" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106110/</t>
-        </is>
-      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -8747,11 +7203,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E308" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106111/</t>
-        </is>
-      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -8774,11 +7225,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E309" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106112/</t>
-        </is>
-      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -8801,11 +7247,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E310" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106113/</t>
-        </is>
-      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -8828,11 +7269,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E311" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106114/</t>
-        </is>
-      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -8855,11 +7291,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E312" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106115/</t>
-        </is>
-      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -8882,11 +7313,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E313" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106116/</t>
-        </is>
-      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -8909,11 +7335,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E314" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106117/</t>
-        </is>
-      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -8936,11 +7357,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E315" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106118/</t>
-        </is>
-      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -8963,11 +7379,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E316" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/HAVISHMATHIS/</t>
-        </is>
-      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -8990,11 +7401,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E317" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106120/</t>
-        </is>
-      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -9017,11 +7423,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E318" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Jai_Ganesh_I/</t>
-        </is>
-      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -9044,11 +7445,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E319" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106121/</t>
-        </is>
-      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -9071,11 +7467,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E320" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106122/</t>
-        </is>
-      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -9098,11 +7489,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E321" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106123/</t>
-        </is>
-      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -9125,11 +7511,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E322" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106124/</t>
-        </is>
-      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -9152,11 +7533,6 @@
           <t>ECE B</t>
         </is>
       </c>
-      <c r="E323" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/922525106126/</t>
-        </is>
-      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -9179,11 +7555,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E324" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/janani_asohkan/</t>
-        </is>
-      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -9206,11 +7577,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E325" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/jashvanth2007/</t>
-        </is>
-      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -9233,11 +7599,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E326" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/jayasakthi_25/</t>
-        </is>
-      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -9260,11 +7621,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E327" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/jeevanbala142008/</t>
-        </is>
-      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -9287,11 +7643,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E328" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/dharshanjeeva/</t>
-        </is>
-      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -9314,11 +7665,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E329" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/jeevanaa_174_/</t>
-        </is>
-      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -9341,11 +7687,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E330" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Jerry2008/</t>
-        </is>
-      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -9368,11 +7709,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E331" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Joshi_666/</t>
-        </is>
-      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -9395,11 +7731,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E332" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Jothiharshan16/</t>
-        </is>
-      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -9422,11 +7753,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E333" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Jothi-/</t>
-        </is>
-      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -9449,11 +7775,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E334" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/_kamalini_/</t>
-        </is>
-      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -9476,11 +7797,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E335" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/26kanishka/</t>
-        </is>
-      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -9503,11 +7819,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E336" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/kanithraakila/</t>
-        </is>
-      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -9530,11 +7841,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E337" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Karishma_m_08/</t>
-        </is>
-      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -9557,11 +7863,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E338" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/karmukilan567/</t>
-        </is>
-      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -9584,11 +7885,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E339" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/karshana_234/</t>
-        </is>
-      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -9611,11 +7907,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E340" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Karthi270827/</t>
-        </is>
-      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -9638,11 +7929,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E341" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/kavimalar08/</t>
-        </is>
-      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -9665,11 +7951,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E342" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/KAVIN__26/</t>
-        </is>
-      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -9692,11 +7973,6 @@
           <t>ECE A</t>
         </is>
       </c>
-      <c r="E343" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/AjaykumarAL/</t>
-        </is>
-      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -9719,11 +7995,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E344" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/kavinleet/</t>
-        </is>
-      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -9746,11 +8017,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E345" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/_kavipriya_16/</t>
-        </is>
-      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -9773,11 +8039,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E346" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/KAVI_RAVI/</t>
-        </is>
-      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -9800,11 +8061,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E347" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/kavi12d/</t>
-        </is>
-      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -9827,11 +8083,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E348" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/mahi20_/</t>
-        </is>
-      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -9854,11 +8105,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E349" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/itzz__kavya02/</t>
-        </is>
-      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -9881,11 +8127,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E350" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/27kayalvizhi/</t>
-        </is>
-      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -9908,11 +8149,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E351" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/keerthana_19selvam/</t>
-        </is>
-      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -9935,11 +8171,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E352" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/KESAVINI892/</t>
-        </is>
-      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -9962,11 +8193,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E353" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/kiruthika_selvanathan05092007/</t>
-        </is>
-      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -9989,11 +8215,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E354" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/kohul_v/</t>
-        </is>
-      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -10016,11 +8237,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E355" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/kowshikm23/</t>
-        </is>
-      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -10043,11 +8259,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E356" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/kowshik_rk_/</t>
-        </is>
-      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -10070,11 +8281,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E357" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Kowshika08/</t>
-        </is>
-      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -10097,11 +8303,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E358" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/kowshika_moorthi/</t>
-        </is>
-      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -10124,11 +8325,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E359" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/KOWSHIKAN-PALANISAMY/</t>
-        </is>
-      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -10151,11 +8347,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E360" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Harjit_Vasan/</t>
-        </is>
-      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -10178,11 +8369,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E361" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/LOHITH1206/</t>
-        </is>
-      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -10205,11 +8391,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E362" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Sanjay_Sakthivel-2/</t>
-        </is>
-      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -10232,11 +8413,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E363" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/SATHYAPRAKASAM__7/</t>
-        </is>
-      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -10259,11 +8435,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E364" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/kanishkumar2008/</t>
-        </is>
-      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -10286,11 +8457,6 @@
           <t>ECE C</t>
         </is>
       </c>
-      <c r="E365" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Kishore9225/</t>
-        </is>
-      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -10313,11 +8479,6 @@
           <t>ECE D</t>
         </is>
       </c>
-      <c r="E366" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Nethra777/</t>
-        </is>
-      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -10340,11 +8501,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E367" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/sanjevi007/</t>
-        </is>
-      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -10367,11 +8523,6 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E368" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/arunkumar1004/</t>
-        </is>
-      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -10394,14 +8545,8 @@
           <t>ECE E</t>
         </is>
       </c>
-      <c r="E369" t="inlineStr">
-        <is>
-          <t>https://leetcode.com/u/Rithik2008/</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E369"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>